<commit_message>
Forbid confidence levels below 50.
</commit_message>
<xml_diff>
--- a/inst/extdata/topics.xlsx
+++ b/inst/extdata/topics.xlsx
@@ -430,10 +430,10 @@
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E2" t="n">
-        <v>0.08</v>
+        <v>0.57</v>
       </c>
     </row>
     <row r="3">
@@ -447,10 +447,10 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="4">
@@ -464,10 +464,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E4" t="n">
-        <v>0.85</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E5" t="n">
         <v>0.02</v>
@@ -498,10 +498,10 @@
         <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E6" t="n">
-        <v>0.05</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="7">
@@ -515,10 +515,10 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E7" t="n">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="8">
@@ -532,10 +532,10 @@
         <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E8" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="9">
@@ -549,10 +549,10 @@
         <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E9" t="n">
-        <v>0.18</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="10">
@@ -566,10 +566,10 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E10" t="n">
-        <v>0.02</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="11">
@@ -583,10 +583,10 @@
         <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E11" t="n">
-        <v>0.67</v>
+        <v>0.36</v>
       </c>
     </row>
     <row r="12">
@@ -600,10 +600,10 @@
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E12" t="n">
-        <v>0.43</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="13">
@@ -617,10 +617,10 @@
         <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E13" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="14">
@@ -634,10 +634,10 @@
         <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E14" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="15">
@@ -651,10 +651,10 @@
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E15" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="16">
@@ -668,10 +668,10 @@
         <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="E16" t="n">
-        <v>0.18</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="17">
@@ -685,10 +685,10 @@
         <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E17" t="n">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="18">
@@ -702,10 +702,10 @@
         <v>8</v>
       </c>
       <c r="D18" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="19">
@@ -719,10 +719,10 @@
         <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E19" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="20">
@@ -736,10 +736,10 @@
         <v>10</v>
       </c>
       <c r="D20" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E20" t="n">
-        <v>0.05</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="21">
@@ -753,7 +753,7 @@
         <v>11</v>
       </c>
       <c r="D21" t="n">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="E21" t="n">
         <v>0.08</v>
@@ -770,10 +770,10 @@
         <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E22" t="n">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="23">
@@ -787,10 +787,10 @@
         <v>8</v>
       </c>
       <c r="D23" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E23" t="n">
-        <v>0.21</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="24">
@@ -804,10 +804,10 @@
         <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E24" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="25">
@@ -821,10 +821,10 @@
         <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E25" t="n">
-        <v>0.01</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="26">
@@ -838,10 +838,10 @@
         <v>11</v>
       </c>
       <c r="D26" t="n">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="E26" t="n">
-        <v>0.45</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="27">
@@ -855,10 +855,10 @@
         <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E27" t="n">
-        <v>0.37</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="28">
@@ -872,10 +872,10 @@
         <v>8</v>
       </c>
       <c r="D28" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E28" t="n">
-        <v>0.06</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="29">
@@ -889,10 +889,10 @@
         <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E29" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="30">
@@ -906,10 +906,10 @@
         <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E30" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -923,10 +923,10 @@
         <v>11</v>
       </c>
       <c r="D31" t="n">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="E31" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="32">
@@ -940,10 +940,10 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E32" t="n">
-        <v>0.43</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="33">
@@ -957,10 +957,10 @@
         <v>8</v>
       </c>
       <c r="D33" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E33" t="n">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="34">
@@ -974,10 +974,10 @@
         <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="35">
@@ -991,10 +991,10 @@
         <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="36">
@@ -1008,10 +1008,10 @@
         <v>11</v>
       </c>
       <c r="D36" t="n">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="E36" t="n">
-        <v>0.22</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="37">
@@ -1025,10 +1025,10 @@
         <v>7</v>
       </c>
       <c r="D37" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E37" t="n">
-        <v>0.01</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="38">
@@ -1042,10 +1042,10 @@
         <v>8</v>
       </c>
       <c r="D38" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E38" t="n">
-        <v>0.29</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="39">
@@ -1059,10 +1059,10 @@
         <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E39" t="n">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="40">
@@ -1076,10 +1076,10 @@
         <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E40" t="n">
-        <v>0.5</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="41">
@@ -1093,10 +1093,10 @@
         <v>11</v>
       </c>
       <c r="D41" t="n">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="E41" t="n">
-        <v>0.12</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="42">
@@ -1110,10 +1110,10 @@
         <v>7</v>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E42" t="n">
-        <v>0.13</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="43">
@@ -1127,10 +1127,10 @@
         <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E43" t="n">
-        <v>0.01</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="44">
@@ -1144,10 +1144,10 @@
         <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E44" t="n">
-        <v>0.58</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="45">
@@ -1161,10 +1161,10 @@
         <v>10</v>
       </c>
       <c r="D45" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E45" t="n">
-        <v>0.24</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="46">
@@ -1178,10 +1178,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E46" t="n">
-        <v>0.04</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="47">
@@ -1195,10 +1195,10 @@
         <v>7</v>
       </c>
       <c r="D47" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E47" t="n">
-        <v>0.18</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="48">
@@ -1212,10 +1212,10 @@
         <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E48" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="49">
@@ -1229,10 +1229,10 @@
         <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E49" t="n">
-        <v>0.27</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="50">
@@ -1246,10 +1246,10 @@
         <v>10</v>
       </c>
       <c r="D50" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E50" t="n">
-        <v>0.23</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="51">
@@ -1263,10 +1263,10 @@
         <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E51" t="n">
-        <v>0.17</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="52">
@@ -1280,10 +1280,10 @@
         <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="E52" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="53">
@@ -1297,10 +1297,10 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="54">
@@ -1314,10 +1314,10 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="E54" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="55">
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="E55" t="n">
-        <v>0.44</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="56">
@@ -1348,10 +1348,10 @@
         <v>11</v>
       </c>
       <c r="D56" t="n">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="E56" t="n">
-        <v>0.31</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="57">
@@ -1365,10 +1365,10 @@
         <v>7</v>
       </c>
       <c r="D57" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E57" t="n">
-        <v>0.44</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="58">
@@ -1382,10 +1382,10 @@
         <v>8</v>
       </c>
       <c r="D58" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E58" t="n">
-        <v>0.05</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="59">
@@ -1399,10 +1399,10 @@
         <v>9</v>
       </c>
       <c r="D59" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E59" t="n">
-        <v>0.26</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="60">
@@ -1416,10 +1416,10 @@
         <v>10</v>
       </c>
       <c r="D60" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E60" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="61">
@@ -1433,10 +1433,10 @@
         <v>11</v>
       </c>
       <c r="D61" t="n">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="E61" t="n">
-        <v>0.17</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="62">
@@ -1450,10 +1450,10 @@
         <v>7</v>
       </c>
       <c r="D62" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E62" t="n">
-        <v>0.07</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="63">
@@ -1467,10 +1467,10 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E63" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1484,10 +1484,10 @@
         <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E64" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="65">
@@ -1501,10 +1501,10 @@
         <v>10</v>
       </c>
       <c r="D65" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E65" t="n">
-        <v>0.32</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="66">
@@ -1518,10 +1518,10 @@
         <v>11</v>
       </c>
       <c r="D66" t="n">
-        <v>55</v>
+        <v>91</v>
       </c>
       <c r="E66" t="n">
-        <v>0.43</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="67">
@@ -1535,10 +1535,10 @@
         <v>7</v>
       </c>
       <c r="D67" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E67" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="68">
@@ -1552,10 +1552,10 @@
         <v>8</v>
       </c>
       <c r="D68" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E68" t="n">
-        <v>0.48</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="69">
@@ -1569,10 +1569,10 @@
         <v>9</v>
       </c>
       <c r="D69" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E69" t="n">
-        <v>0.05</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="70">
@@ -1586,10 +1586,10 @@
         <v>10</v>
       </c>
       <c r="D70" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E70" t="n">
-        <v>0.03</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="71">
@@ -1603,10 +1603,10 @@
         <v>11</v>
       </c>
       <c r="D71" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E71" t="n">
-        <v>0.32</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="72">
@@ -1620,10 +1620,10 @@
         <v>7</v>
       </c>
       <c r="D72" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="E72" t="n">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="73">
@@ -1637,10 +1637,10 @@
         <v>8</v>
       </c>
       <c r="D73" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="E73" t="n">
-        <v>0.27</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="74">
@@ -1654,10 +1654,10 @@
         <v>9</v>
       </c>
       <c r="D74" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="E74" t="n">
-        <v>0.35</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="75">
@@ -1671,10 +1671,10 @@
         <v>10</v>
       </c>
       <c r="D75" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="E75" t="n">
-        <v>0.13</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="76">
@@ -1688,10 +1688,10 @@
         <v>11</v>
       </c>
       <c r="D76" t="n">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="E76" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="77">
@@ -1705,10 +1705,10 @@
         <v>7</v>
       </c>
       <c r="D77" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E77" t="n">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="78">
@@ -1722,10 +1722,10 @@
         <v>8</v>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E78" t="n">
-        <v>0.22</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="79">
@@ -1739,10 +1739,10 @@
         <v>9</v>
       </c>
       <c r="D79" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E79" t="n">
-        <v>0.19</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="80">
@@ -1756,10 +1756,10 @@
         <v>10</v>
       </c>
       <c r="D80" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E80" t="n">
-        <v>0.36</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="81">
@@ -1773,10 +1773,10 @@
         <v>11</v>
       </c>
       <c r="D81" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E81" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="82">
@@ -1790,10 +1790,10 @@
         <v>7</v>
       </c>
       <c r="D82" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="E82" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="83">
@@ -1807,10 +1807,10 @@
         <v>8</v>
       </c>
       <c r="D83" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="E83" t="n">
-        <v>0.01</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="84">
@@ -1824,10 +1824,10 @@
         <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="E84" t="n">
-        <v>0.31</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="85">
@@ -1841,10 +1841,10 @@
         <v>10</v>
       </c>
       <c r="D85" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="E85" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="86">
@@ -1858,10 +1858,10 @@
         <v>11</v>
       </c>
       <c r="D86" t="n">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="E86" t="n">
-        <v>0.23</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="87">
@@ -1875,10 +1875,10 @@
         <v>7</v>
       </c>
       <c r="D87" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E87" t="n">
-        <v>0.34</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="88">
@@ -1892,10 +1892,10 @@
         <v>8</v>
       </c>
       <c r="D88" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E88" t="n">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="89">
@@ -1909,10 +1909,10 @@
         <v>9</v>
       </c>
       <c r="D89" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E89" t="n">
-        <v>0.25</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="90">
@@ -1926,10 +1926,10 @@
         <v>10</v>
       </c>
       <c r="D90" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E90" t="n">
-        <v>0.13</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="91">
@@ -1943,10 +1943,10 @@
         <v>11</v>
       </c>
       <c r="D91" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E91" t="n">
-        <v>0.19</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="92">
@@ -1960,10 +1960,10 @@
         <v>7</v>
       </c>
       <c r="D92" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E92" t="n">
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="93">
@@ -1977,10 +1977,10 @@
         <v>8</v>
       </c>
       <c r="D93" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E93" t="n">
-        <v>0.33</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="94">
@@ -1994,10 +1994,10 @@
         <v>9</v>
       </c>
       <c r="D94" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E94" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="95">
@@ -2011,10 +2011,10 @@
         <v>10</v>
       </c>
       <c r="D95" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E95" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="96">
@@ -2028,10 +2028,10 @@
         <v>11</v>
       </c>
       <c r="D96" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E96" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="97">
@@ -2045,10 +2045,10 @@
         <v>7</v>
       </c>
       <c r="D97" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E97" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="98">
@@ -2062,10 +2062,10 @@
         <v>8</v>
       </c>
       <c r="D98" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E98" t="n">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="99">
@@ -2079,10 +2079,10 @@
         <v>9</v>
       </c>
       <c r="D99" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E99" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="100">
@@ -2096,10 +2096,10 @@
         <v>10</v>
       </c>
       <c r="D100" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E100" t="n">
-        <v>0.15</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="101">
@@ -2113,10 +2113,10 @@
         <v>11</v>
       </c>
       <c r="D101" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E101" t="n">
-        <v>0.3</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="102">
@@ -2130,10 +2130,10 @@
         <v>7</v>
       </c>
       <c r="D102" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E102" t="n">
-        <v>0.19</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="103">
@@ -2147,10 +2147,10 @@
         <v>8</v>
       </c>
       <c r="D103" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E103" t="n">
-        <v>0.01</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="104">
@@ -2164,10 +2164,10 @@
         <v>9</v>
       </c>
       <c r="D104" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E104" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="105">
@@ -2181,10 +2181,10 @@
         <v>10</v>
       </c>
       <c r="D105" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E105" t="n">
-        <v>0.01</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="106">
@@ -2198,10 +2198,10 @@
         <v>11</v>
       </c>
       <c r="D106" t="n">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="E106" t="n">
-        <v>0.63</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="107">
@@ -2215,10 +2215,10 @@
         <v>7</v>
       </c>
       <c r="D107" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E107" t="n">
-        <v>0.13</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="108">
@@ -2232,10 +2232,10 @@
         <v>8</v>
       </c>
       <c r="D108" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E108" t="n">
-        <v>0.34</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="109">
@@ -2249,10 +2249,10 @@
         <v>9</v>
       </c>
       <c r="D109" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E109" t="n">
-        <v>0.47</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="110">
@@ -2266,10 +2266,10 @@
         <v>10</v>
       </c>
       <c r="D110" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E110" t="n">
-        <v>0.04</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="111">
@@ -2283,10 +2283,10 @@
         <v>11</v>
       </c>
       <c r="D111" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E111" t="n">
-        <v>0.02</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="112">
@@ -2300,10 +2300,10 @@
         <v>7</v>
       </c>
       <c r="D112" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E112" t="n">
-        <v>0.37</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="113">
@@ -2317,10 +2317,10 @@
         <v>8</v>
       </c>
       <c r="D113" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E113" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="114">
@@ -2334,10 +2334,10 @@
         <v>9</v>
       </c>
       <c r="D114" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E114" t="n">
-        <v>0.52</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="115">
@@ -2351,10 +2351,10 @@
         <v>10</v>
       </c>
       <c r="D115" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E115" t="n">
-        <v>0.03</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="116">
@@ -2368,10 +2368,10 @@
         <v>11</v>
       </c>
       <c r="D116" t="n">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="E116" t="n">
-        <v>0</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="117">
@@ -2385,10 +2385,10 @@
         <v>7</v>
       </c>
       <c r="D117" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E117" t="n">
-        <v>0.07</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="118">
@@ -2402,10 +2402,10 @@
         <v>8</v>
       </c>
       <c r="D118" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E118" t="n">
-        <v>0.35</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="119">
@@ -2419,10 +2419,10 @@
         <v>9</v>
       </c>
       <c r="D119" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E119" t="n">
-        <v>0.45</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="120">
@@ -2436,10 +2436,10 @@
         <v>10</v>
       </c>
       <c r="D120" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E120" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="121">
@@ -2453,10 +2453,10 @@
         <v>11</v>
       </c>
       <c r="D121" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E121" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2498,10 +2498,10 @@
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E2" t="n">
-        <v>0.09</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="3">
@@ -2515,10 +2515,10 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E3" t="n">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="4">
@@ -2532,10 +2532,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E4" t="n">
-        <v>0.11</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="5">
@@ -2549,10 +2549,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E5" t="n">
-        <v>0.59</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="6">
@@ -2566,7 +2566,7 @@
         <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -2583,10 +2583,10 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="E7" t="n">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="8">
@@ -2600,10 +2600,10 @@
         <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="E8" t="n">
-        <v>0.05</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="9">
@@ -2617,10 +2617,10 @@
         <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="E9" t="n">
-        <v>0.33</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="10">
@@ -2634,10 +2634,10 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="E10" t="n">
-        <v>0.24</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="11">
@@ -2651,10 +2651,10 @@
         <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="E11" t="n">
-        <v>0.29</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="12">
@@ -2668,10 +2668,10 @@
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E12" t="n">
-        <v>0.19</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13">
@@ -2685,10 +2685,10 @@
         <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E13" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2702,10 +2702,10 @@
         <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="15">
@@ -2719,10 +2719,10 @@
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E15" t="n">
-        <v>0.47</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="16">
@@ -2736,10 +2736,10 @@
         <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E16" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="17">
@@ -2753,10 +2753,10 @@
         <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E17" t="n">
-        <v>0.02</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="18">
@@ -2770,10 +2770,10 @@
         <v>8</v>
       </c>
       <c r="D18" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E18" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="19">
@@ -2787,10 +2787,10 @@
         <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E19" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="20">
@@ -2804,10 +2804,10 @@
         <v>10</v>
       </c>
       <c r="D20" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E20" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="21">
@@ -2821,10 +2821,10 @@
         <v>11</v>
       </c>
       <c r="D21" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E21" t="n">
-        <v>0.37</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="22">
@@ -2838,10 +2838,10 @@
         <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E22" t="n">
-        <v>0.31</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="23">
@@ -2855,10 +2855,10 @@
         <v>8</v>
       </c>
       <c r="D23" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E23" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="24">
@@ -2872,10 +2872,10 @@
         <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E24" t="n">
-        <v>0.09</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="25">
@@ -2889,10 +2889,10 @@
         <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E25" t="n">
-        <v>0.17</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="26">
@@ -2906,10 +2906,10 @@
         <v>11</v>
       </c>
       <c r="D26" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E26" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="27">
@@ -2923,10 +2923,10 @@
         <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E27" t="n">
-        <v>0.03</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="28">
@@ -2940,10 +2940,10 @@
         <v>8</v>
       </c>
       <c r="D28" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E28" t="n">
-        <v>0.73</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="29">
@@ -2957,10 +2957,10 @@
         <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E29" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="30">
@@ -2974,10 +2974,10 @@
         <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E30" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="31">
@@ -2991,10 +2991,10 @@
         <v>11</v>
       </c>
       <c r="D31" t="n">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="E31" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="32">
@@ -3008,10 +3008,10 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E32" t="n">
-        <v>0.21</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="33">
@@ -3025,10 +3025,10 @@
         <v>8</v>
       </c>
       <c r="D33" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E33" t="n">
-        <v>0.02</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="34">
@@ -3042,10 +3042,10 @@
         <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E34" t="n">
-        <v>0.09</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="35">
@@ -3059,10 +3059,10 @@
         <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E35" t="n">
-        <v>0.42</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="36">
@@ -3076,10 +3076,10 @@
         <v>11</v>
       </c>
       <c r="D36" t="n">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="E36" t="n">
-        <v>0.26</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="37">
@@ -3093,10 +3093,10 @@
         <v>7</v>
       </c>
       <c r="D37" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E37" t="n">
-        <v>0.53</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="38">
@@ -3110,10 +3110,10 @@
         <v>8</v>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E38" t="n">
-        <v>0.02</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="39">
@@ -3127,10 +3127,10 @@
         <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E39" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="40">
@@ -3144,10 +3144,10 @@
         <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E40" t="n">
-        <v>0.4</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="41">
@@ -3161,10 +3161,10 @@
         <v>11</v>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="E41" t="n">
-        <v>0.01</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="42">
@@ -3178,10 +3178,10 @@
         <v>7</v>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E42" t="n">
-        <v>0.55</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="43">
@@ -3195,10 +3195,10 @@
         <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E43" t="n">
-        <v>0.03</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="44">
@@ -3212,7 +3212,7 @@
         <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E44" t="n">
         <v>0.01</v>
@@ -3229,10 +3229,10 @@
         <v>10</v>
       </c>
       <c r="D45" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E45" t="n">
-        <v>0.11</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="46">
@@ -3246,10 +3246,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="47">
@@ -3263,10 +3263,10 @@
         <v>7</v>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E47" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="48">
@@ -3280,10 +3280,10 @@
         <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="49">
@@ -3297,10 +3297,10 @@
         <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E49" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="50">
@@ -3314,10 +3314,10 @@
         <v>10</v>
       </c>
       <c r="D50" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E50" t="n">
-        <v>0.16</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="51">
@@ -3331,10 +3331,10 @@
         <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E51" t="n">
-        <v>0.68</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="52">
@@ -3348,10 +3348,10 @@
         <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E52" t="n">
-        <v>0.47</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="53">
@@ -3365,10 +3365,10 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E53" t="n">
-        <v>0.04</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="54">
@@ -3382,10 +3382,10 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="55">
@@ -3399,10 +3399,10 @@
         <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E55" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="56">
@@ -3416,10 +3416,10 @@
         <v>11</v>
       </c>
       <c r="D56" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E56" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="57">
@@ -3433,10 +3433,10 @@
         <v>7</v>
       </c>
       <c r="D57" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E57" t="n">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="58">
@@ -3450,10 +3450,10 @@
         <v>8</v>
       </c>
       <c r="D58" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E58" t="n">
-        <v>0.19</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="59">
@@ -3467,10 +3467,10 @@
         <v>9</v>
       </c>
       <c r="D59" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E59" t="n">
-        <v>0.28</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="60">
@@ -3484,7 +3484,7 @@
         <v>10</v>
       </c>
       <c r="D60" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E60" t="n">
         <v>0.34</v>
@@ -3501,10 +3501,10 @@
         <v>11</v>
       </c>
       <c r="D61" t="n">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E61" t="n">
-        <v>0.08</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="62">
@@ -3518,10 +3518,10 @@
         <v>7</v>
       </c>
       <c r="D62" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E62" t="n">
-        <v>0.28</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="63">
@@ -3535,10 +3535,10 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E63" t="n">
-        <v>0.04</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="64">
@@ -3552,10 +3552,10 @@
         <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E64" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="65">
@@ -3569,10 +3569,10 @@
         <v>10</v>
       </c>
       <c r="D65" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E65" t="n">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="66">
@@ -3586,10 +3586,10 @@
         <v>11</v>
       </c>
       <c r="D66" t="n">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E66" t="n">
-        <v>0.47</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="67">
@@ -3603,10 +3603,10 @@
         <v>7</v>
       </c>
       <c r="D67" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E67" t="n">
-        <v>0.12</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="68">
@@ -3620,10 +3620,10 @@
         <v>8</v>
       </c>
       <c r="D68" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E68" t="n">
-        <v>0.27</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="69">
@@ -3637,10 +3637,10 @@
         <v>9</v>
       </c>
       <c r="D69" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E69" t="n">
-        <v>0.02</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="70">
@@ -3654,10 +3654,10 @@
         <v>10</v>
       </c>
       <c r="D70" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E70" t="n">
-        <v>0.4</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="71">
@@ -3671,10 +3671,10 @@
         <v>11</v>
       </c>
       <c r="D71" t="n">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="E71" t="n">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="72">
@@ -3688,10 +3688,10 @@
         <v>7</v>
       </c>
       <c r="D72" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E72" t="n">
-        <v>0.05</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="73">
@@ -3705,10 +3705,10 @@
         <v>8</v>
       </c>
       <c r="D73" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E73" t="n">
-        <v>0.02</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="74">
@@ -3722,10 +3722,10 @@
         <v>9</v>
       </c>
       <c r="D74" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E74" t="n">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="75">
@@ -3739,10 +3739,10 @@
         <v>10</v>
       </c>
       <c r="D75" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E75" t="n">
-        <v>0.08</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="76">
@@ -3756,10 +3756,10 @@
         <v>11</v>
       </c>
       <c r="D76" t="n">
-        <v>15</v>
+        <v>71</v>
       </c>
       <c r="E76" t="n">
-        <v>0.53</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="77">
@@ -3773,10 +3773,10 @@
         <v>7</v>
       </c>
       <c r="D77" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E77" t="n">
-        <v>0.32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -3790,10 +3790,10 @@
         <v>8</v>
       </c>
       <c r="D78" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E78" t="n">
-        <v>0.44</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="79">
@@ -3807,10 +3807,10 @@
         <v>9</v>
       </c>
       <c r="D79" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E79" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="80">
@@ -3824,10 +3824,10 @@
         <v>10</v>
       </c>
       <c r="D80" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E80" t="n">
-        <v>0.09</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="81">
@@ -3841,10 +3841,10 @@
         <v>11</v>
       </c>
       <c r="D81" t="n">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="E81" t="n">
-        <v>0.02</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="82">
@@ -3858,10 +3858,10 @@
         <v>7</v>
       </c>
       <c r="D82" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E82" t="n">
-        <v>0.34</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="83">
@@ -3875,7 +3875,7 @@
         <v>8</v>
       </c>
       <c r="D83" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E83" t="n">
         <v>0.04</v>
@@ -3892,10 +3892,10 @@
         <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E84" t="n">
-        <v>0.3</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="85">
@@ -3909,10 +3909,10 @@
         <v>10</v>
       </c>
       <c r="D85" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E85" t="n">
-        <v>0.03</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="86">
@@ -3926,10 +3926,10 @@
         <v>11</v>
       </c>
       <c r="D86" t="n">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="E86" t="n">
-        <v>0.29</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="87">
@@ -3943,10 +3943,10 @@
         <v>7</v>
       </c>
       <c r="D87" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E87" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="88">
@@ -3960,10 +3960,10 @@
         <v>8</v>
       </c>
       <c r="D88" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E88" t="n">
-        <v>0.09</v>
+        <v>0.56</v>
       </c>
     </row>
     <row r="89">
@@ -3977,10 +3977,10 @@
         <v>9</v>
       </c>
       <c r="D89" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E89" t="n">
-        <v>0.07</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="90">
@@ -3994,10 +3994,10 @@
         <v>10</v>
       </c>
       <c r="D90" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E90" t="n">
-        <v>0.75</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="91">
@@ -4011,10 +4011,10 @@
         <v>11</v>
       </c>
       <c r="D91" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="E91" t="n">
-        <v>0.01</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="92">
@@ -4028,10 +4028,10 @@
         <v>7</v>
       </c>
       <c r="D92" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E92" t="n">
-        <v>0.23</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="93">
@@ -4045,10 +4045,10 @@
         <v>8</v>
       </c>
       <c r="D93" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E93" t="n">
-        <v>0.49</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="94">
@@ -4062,10 +4062,10 @@
         <v>9</v>
       </c>
       <c r="D94" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E94" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="95">
@@ -4079,10 +4079,10 @@
         <v>10</v>
       </c>
       <c r="D95" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E95" t="n">
-        <v>0.17</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="96">
@@ -4096,10 +4096,10 @@
         <v>11</v>
       </c>
       <c r="D96" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E96" t="n">
-        <v>0.09</v>
+        <v>0.56</v>
       </c>
     </row>
     <row r="97">
@@ -4113,10 +4113,10 @@
         <v>7</v>
       </c>
       <c r="D97" t="n">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E97" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="98">
@@ -4130,10 +4130,10 @@
         <v>8</v>
       </c>
       <c r="D98" t="n">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E98" t="n">
-        <v>0.09</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="99">
@@ -4147,10 +4147,10 @@
         <v>9</v>
       </c>
       <c r="D99" t="n">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E99" t="n">
-        <v>0.52</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="100">
@@ -4164,10 +4164,10 @@
         <v>10</v>
       </c>
       <c r="D100" t="n">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E100" t="n">
-        <v>0.09</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="101">
@@ -4181,10 +4181,10 @@
         <v>11</v>
       </c>
       <c r="D101" t="n">
-        <v>40</v>
+        <v>91</v>
       </c>
       <c r="E101" t="n">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
     </row>
   </sheetData>
@@ -4226,10 +4226,10 @@
         <v>7</v>
       </c>
       <c r="D2" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="3">
@@ -4243,10 +4243,10 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -4260,10 +4260,10 @@
         <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="5">
@@ -4277,10 +4277,10 @@
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E5" t="n">
-        <v>0.87</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="6">
@@ -4294,10 +4294,10 @@
         <v>11</v>
       </c>
       <c r="D6" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E6" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -4311,10 +4311,10 @@
         <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="E7" t="n">
-        <v>0.11</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="8">
@@ -4328,10 +4328,10 @@
         <v>8</v>
       </c>
       <c r="D8" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="E8" t="n">
-        <v>0.09</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="9">
@@ -4345,10 +4345,10 @@
         <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="E9" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="10">
@@ -4362,10 +4362,10 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="E10" t="n">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11">
@@ -4379,10 +4379,10 @@
         <v>11</v>
       </c>
       <c r="D11" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="E11" t="n">
-        <v>0.54</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="12">
@@ -4396,7 +4396,7 @@
         <v>7</v>
       </c>
       <c r="D12" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="E12" t="n">
         <v>0.59</v>
@@ -4413,10 +4413,10 @@
         <v>8</v>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="E13" t="n">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="14">
@@ -4430,10 +4430,10 @@
         <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="E14" t="n">
-        <v>0.11</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="15">
@@ -4447,10 +4447,10 @@
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="16">
@@ -4464,10 +4464,10 @@
         <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>15</v>
+        <v>91</v>
       </c>
       <c r="E16" t="n">
-        <v>0.22</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="17">
@@ -4481,10 +4481,10 @@
         <v>7</v>
       </c>
       <c r="D17" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="E17" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="18">
@@ -4498,10 +4498,10 @@
         <v>8</v>
       </c>
       <c r="D18" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="E18" t="n">
-        <v>0.38</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="19">
@@ -4515,10 +4515,10 @@
         <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="E19" t="n">
-        <v>0.16</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="20">
@@ -4532,10 +4532,10 @@
         <v>10</v>
       </c>
       <c r="D20" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="E20" t="n">
-        <v>0.08</v>
+        <v>0.27</v>
       </c>
     </row>
     <row r="21">
@@ -4549,7 +4549,7 @@
         <v>11</v>
       </c>
       <c r="D21" t="n">
-        <v>25</v>
+        <v>96</v>
       </c>
       <c r="E21" t="n">
         <v>0.12</v>
@@ -4566,10 +4566,10 @@
         <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>100</v>
+        <v>61</v>
       </c>
       <c r="E22" t="n">
-        <v>0.42</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="23">
@@ -4583,10 +4583,10 @@
         <v>8</v>
       </c>
       <c r="D23" t="n">
-        <v>100</v>
+        <v>61</v>
       </c>
       <c r="E23" t="n">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="24">
@@ -4600,10 +4600,10 @@
         <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>100</v>
+        <v>61</v>
       </c>
       <c r="E24" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="25">
@@ -4617,10 +4617,10 @@
         <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>100</v>
+        <v>61</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="26">
@@ -4634,10 +4634,10 @@
         <v>11</v>
       </c>
       <c r="D26" t="n">
-        <v>100</v>
+        <v>61</v>
       </c>
       <c r="E26" t="n">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="27">
@@ -4651,10 +4651,10 @@
         <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E27" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="28">
@@ -4668,10 +4668,10 @@
         <v>8</v>
       </c>
       <c r="D28" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E28" t="n">
-        <v>0.3</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="29">
@@ -4685,10 +4685,10 @@
         <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E29" t="n">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="30">
@@ -4702,10 +4702,10 @@
         <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E30" t="n">
-        <v>0.06</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="31">
@@ -4719,10 +4719,10 @@
         <v>11</v>
       </c>
       <c r="D31" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E31" t="n">
-        <v>0.32</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="32">
@@ -4736,10 +4736,10 @@
         <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E32" t="n">
-        <v>0.04</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="33">
@@ -4753,10 +4753,10 @@
         <v>8</v>
       </c>
       <c r="D33" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E33" t="n">
-        <v>0.45</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="34">
@@ -4770,10 +4770,10 @@
         <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E34" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="35">
@@ -4787,10 +4787,10 @@
         <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E35" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="36">
@@ -4804,10 +4804,10 @@
         <v>11</v>
       </c>
       <c r="D36" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E36" t="n">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="37">
@@ -4821,10 +4821,10 @@
         <v>7</v>
       </c>
       <c r="D37" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E37" t="n">
-        <v>0.24</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="38">
@@ -4838,10 +4838,10 @@
         <v>8</v>
       </c>
       <c r="D38" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E38" t="n">
-        <v>0.31</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="39">
@@ -4855,10 +4855,10 @@
         <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E39" t="n">
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="40">
@@ -4872,10 +4872,10 @@
         <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E40" t="n">
-        <v>0.02</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="41">
@@ -4889,10 +4889,10 @@
         <v>11</v>
       </c>
       <c r="D41" t="n">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="E41" t="n">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="42">
@@ -4906,10 +4906,10 @@
         <v>7</v>
       </c>
       <c r="D42" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E42" t="n">
-        <v>0.07</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="43">
@@ -4923,10 +4923,10 @@
         <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E43" t="n">
-        <v>0.12</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="44">
@@ -4940,10 +4940,10 @@
         <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E44" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="45">
@@ -4957,10 +4957,10 @@
         <v>10</v>
       </c>
       <c r="D45" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E45" t="n">
-        <v>0.57</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="46">
@@ -4974,10 +4974,10 @@
         <v>11</v>
       </c>
       <c r="D46" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E46" t="n">
-        <v>0.09</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="47">
@@ -4991,10 +4991,10 @@
         <v>7</v>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E47" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -5008,10 +5008,10 @@
         <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E48" t="n">
-        <v>0.37</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="49">
@@ -5025,10 +5025,10 @@
         <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E49" t="n">
-        <v>0.22</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="50">
@@ -5042,10 +5042,10 @@
         <v>10</v>
       </c>
       <c r="D50" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="51">
@@ -5059,10 +5059,10 @@
         <v>11</v>
       </c>
       <c r="D51" t="n">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="E51" t="n">
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="52">
@@ -5076,10 +5076,10 @@
         <v>7</v>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E52" t="n">
-        <v>0.39</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="53">
@@ -5093,10 +5093,10 @@
         <v>8</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E53" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="54">
@@ -5110,10 +5110,10 @@
         <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E54" t="n">
-        <v>0.01</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="55">
@@ -5127,10 +5127,10 @@
         <v>10</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E55" t="n">
-        <v>0.27</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="56">
@@ -5144,10 +5144,10 @@
         <v>11</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E56" t="n">
-        <v>0.05</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="57">
@@ -5161,10 +5161,10 @@
         <v>7</v>
       </c>
       <c r="D57" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E57" t="n">
-        <v>0.01</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="58">
@@ -5178,10 +5178,10 @@
         <v>8</v>
       </c>
       <c r="D58" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E58" t="n">
-        <v>0.01</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="59">
@@ -5195,10 +5195,10 @@
         <v>9</v>
       </c>
       <c r="D59" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E59" t="n">
-        <v>0.01</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="60">
@@ -5212,10 +5212,10 @@
         <v>10</v>
       </c>
       <c r="D60" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E60" t="n">
-        <v>0.86</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="61">
@@ -5229,10 +5229,10 @@
         <v>11</v>
       </c>
       <c r="D61" t="n">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="E61" t="n">
-        <v>0.11</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="62">
@@ -5246,10 +5246,10 @@
         <v>7</v>
       </c>
       <c r="D62" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E62" t="n">
-        <v>0.15</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="63">
@@ -5263,10 +5263,10 @@
         <v>8</v>
       </c>
       <c r="D63" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E63" t="n">
-        <v>0.22</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="64">
@@ -5280,10 +5280,10 @@
         <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E64" t="n">
-        <v>0.01</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="65">
@@ -5297,10 +5297,10 @@
         <v>10</v>
       </c>
       <c r="D65" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E65" t="n">
-        <v>0.47</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="66">
@@ -5314,10 +5314,10 @@
         <v>11</v>
       </c>
       <c r="D66" t="n">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="E66" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="67">
@@ -5331,10 +5331,10 @@
         <v>7</v>
       </c>
       <c r="D67" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E67" t="n">
-        <v>0.01</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="68">
@@ -5348,10 +5348,10 @@
         <v>8</v>
       </c>
       <c r="D68" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E68" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="69">
@@ -5365,10 +5365,10 @@
         <v>9</v>
       </c>
       <c r="D69" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E69" t="n">
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="70">
@@ -5382,7 +5382,7 @@
         <v>10</v>
       </c>
       <c r="D70" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E70" t="n">
         <v>0.18</v>
@@ -5399,10 +5399,10 @@
         <v>11</v>
       </c>
       <c r="D71" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E71" t="n">
-        <v>0.38</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="72">
@@ -5416,10 +5416,10 @@
         <v>7</v>
       </c>
       <c r="D72" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E72" t="n">
-        <v>0.13</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="73">
@@ -5433,10 +5433,10 @@
         <v>8</v>
       </c>
       <c r="D73" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E73" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="74">
@@ -5450,10 +5450,10 @@
         <v>9</v>
       </c>
       <c r="D74" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E74" t="n">
-        <v>0.34</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="75">
@@ -5467,10 +5467,10 @@
         <v>10</v>
       </c>
       <c r="D75" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E75" t="n">
-        <v>0.49</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="76">
@@ -5484,10 +5484,10 @@
         <v>11</v>
       </c>
       <c r="D76" t="n">
-        <v>55</v>
+        <v>86</v>
       </c>
       <c r="E76" t="n">
-        <v>0.03</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="77">
@@ -5501,10 +5501,10 @@
         <v>7</v>
       </c>
       <c r="D77" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E77" t="n">
-        <v>0.53</v>
+        <v>0.44</v>
       </c>
     </row>
     <row r="78">
@@ -5518,10 +5518,10 @@
         <v>8</v>
       </c>
       <c r="D78" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E78" t="n">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="79">
@@ -5535,10 +5535,10 @@
         <v>9</v>
       </c>
       <c r="D79" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E79" t="n">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="80">
@@ -5552,10 +5552,10 @@
         <v>10</v>
       </c>
       <c r="D80" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E80" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="81">
@@ -5569,10 +5569,10 @@
         <v>11</v>
       </c>
       <c r="D81" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="E81" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="82">
@@ -5586,10 +5586,10 @@
         <v>7</v>
       </c>
       <c r="D82" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E82" t="n">
-        <v>0.28</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="83">
@@ -5603,10 +5603,10 @@
         <v>8</v>
       </c>
       <c r="D83" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E83" t="n">
-        <v>0.24</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="84">
@@ -5620,7 +5620,7 @@
         <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E84" t="n">
         <v>0.09</v>
@@ -5637,10 +5637,10 @@
         <v>10</v>
       </c>
       <c r="D85" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E85" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="86">
@@ -5654,10 +5654,10 @@
         <v>11</v>
       </c>
       <c r="D86" t="n">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="E86" t="n">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="87">
@@ -5671,10 +5671,10 @@
         <v>7</v>
       </c>
       <c r="D87" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E87" t="n">
-        <v>0.32</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="88">
@@ -5688,10 +5688,10 @@
         <v>8</v>
       </c>
       <c r="D88" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E88" t="n">
-        <v>0.05</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="89">
@@ -5705,10 +5705,10 @@
         <v>9</v>
       </c>
       <c r="D89" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E89" t="n">
-        <v>0.46</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="90">
@@ -5722,10 +5722,10 @@
         <v>10</v>
       </c>
       <c r="D90" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E90" t="n">
-        <v>0.02</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="91">
@@ -5739,10 +5739,10 @@
         <v>11</v>
       </c>
       <c r="D91" t="n">
-        <v>35</v>
+        <v>86</v>
       </c>
       <c r="E91" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>